<commit_message>
Use Seaborn and NumPy, remove ';' in dataset
</commit_message>
<xml_diff>
--- a/data/retail_dataset_cleaned.xlsx
+++ b/data/retail_dataset_cleaned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\retail_data_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21A3CC1-7ED1-4AAA-8F6A-4C4EEDEEC741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93AABEB4-6833-49D8-A8D9-90EE28E6E0BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,10 +34,10 @@
     <t>region</t>
   </si>
   <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>City</t>
+    <t>state</t>
+  </si>
+  <si>
+    <t>city</t>
   </si>
   <si>
     <t>product</t>

</xml_diff>